<commit_message>
docs(mejoras): registrar incidencia #13 (scroll del panel) como aplicada
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -922,8 +922,39 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Panel · Conversaciones</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>En el visor de conversaciones, el auto-refresco (cada 5 segundos) tiraba el scroll hasta el fondo, así que no se podía leer hacia arriba: al rato te sacaba del lugar donde estabas leyendo.</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Redibujar el chat solo cuando llegan mensajes nuevos, y bajar al fondo únicamente si el usuario ya estaba abajo o recién abrió esa conversación.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Ahora se puede leer una conversación tranquilo: el panel ya no te tira al final cada 5 segundos y respeta dónde estabas leyendo.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G16"/>
+  <autoFilter ref="A4:G17"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
docs(mejoras): registrar #14 (pedidos reactivados) como aplicada
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -953,8 +953,39 @@
       </c>
       <c r="G17" s="5" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>El agente no podía consultar pedidos de un cliente: cuando se lo pedían, avisaba que 'todavía no está conectado'. Era una capacidad apagada porque la API de Catusita no la exponía.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Catusita implementó el endpoint de pedidos. Se conectó al agente: consulta los pedidos de un cliente por su RUC, con estado del pedido, número de factura SUNAT, estado de despacho (entregado/rechazado) y notas de crédito.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor ya puede preguntar por los pedidos de un cliente y ver en qué estado están, su factura y si se entregaron. Antes esto no estaba disponible.</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G17"/>
+  <autoFilter ref="A4:G18"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
docs(mejoras): registrar #15 (seguimiento de despacho) como aplicada
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -984,8 +984,39 @@
       </c>
       <c r="G18" s="5" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Despacho / Entrega</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>El agente no podía decir si un pedido ya se había entregado ni dar la guía de remisión y las fechas de entrega.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Catusita expuso el endpoint de seguimiento de despacho. Se conectó al agente: por N° de pedido o de factura devuelve si se entregó, la guía de remisión y las fechas de despacho y entrega. La API no permite buscarlo por RUC, así que el agente primero saca los pedidos del cliente y luego consulta el despacho de cada uno.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor ya puede preguntar '¿ya llegó el pedido?' y el agente le dice si se entregó, con qué guía y en qué fecha.</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G18"/>
+  <autoFilter ref="A4:G19"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
docs(mejoras): #16 (sinonimos) y #17 (sku sin stock) aplicadas
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Actualizado: 2026-07-14  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
+          <t>Actualizado: 2026-07-20  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
         </is>
       </c>
     </row>
@@ -1015,8 +1015,70 @@
       </c>
       <c r="G19" s="5" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Buscador de catálogo</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Los vendedores buscan con palabras comunes (amortiguador POSTERIOR, TRASERO, DELANTERO; filtro de HABITÁCULO) pero el catálogo usa abreviaturas (Post, Del) u otros términos, así que da 0 resultados aunque el producto exista. Ejemplo real: 'amortiguador posterior Suzuki Swift' devuelve 0, pero 'amortiguador Post Swift' devuelve 3. Dos vendedores insistieron varias veces y uno nunca encontró su amortiguador.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Agregar un diccionario de sinónimos/abreviaturas al buscador: posterior/trasero → Post, delantero/delantera → Del, habitáculo → cabina/aire, etc. Así la palabra natural del vendedor matchea la abreviatura del catálogo.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor podrá buscar como habla ('amortiguador trasero', 'filtro de habitáculo') y el agente igual encontrará el producto, aunque el catálogo lo tenga abreviado.</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Cuando un SKU existe y tiene precio pero no tiene fila de stock (ej. PP530, que cuesta $55.50), el agente responde 'el sistema no reconoce el código' y entra en un loop pidiendo confirmar el SKU, en vez de decir 'sin stock disponible'. Una vendedora insistió 3 veces con PP530 sin obtener respuesta útil.</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>En la consulta de stock, distinguir 'SKU no existe' de 'SKU válido sin stock'. Si el producto está en el catálogo pero sin fila de stock, responder 'sin stock disponible' (y ofrecer el precio), en vez de tratarlo como código no reconocido y hacer loop.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Cuando un producto existe pero no tiene stock, el agente lo dirá claro ('sin stock disponible') en vez de dar vueltas pidiendo confirmar el código.</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G19"/>
+  <autoFilter ref="A4:G21"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
docs(mejoras): #12 (fotos de productos) pasa a Aplicada - Catusita las expuso
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Actualizado: 2026-07-20  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
+          <t>Actualizado: 2026-07-21 16:06 (hora Perú)  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
         </is>
       </c>
     </row>
@@ -903,22 +903,22 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>A corto plazo, ofrecer una salida clara (dónde ver la imagen). A futuro, conectar las imágenes o fichas técnicas del catálogo cuando estén disponibles.</t>
+          <t>Catusita expuso las imágenes de productos (campo 'images' por artículo). Se conectó al agente: cuando el vendedor pide la foto de un producto por su código, Catu descarga la imagen y se la envía por WhatsApp como foto (no como link).</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>El vendedor podrá ver la foto o ficha técnica del repuesto; hoy el agente no las tiene y solo puede avisar que no están disponibles.</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Rechazado</t>
+          <t>El vendedor ya puede pedir la foto de un producto y Catu se la manda al chat como imagen. Antes se rechazó porque Catusita no las exponía; ahora sí.</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>No es un bug: las imágenes/fichas técnicas no las expone la API de Catusita. Depende de que el proveedor provea ese dato (como pedidos o crédito), no de nuestro código. No hay nada que implementar de nuestro lado por ahora.</t>
+          <t>Estaba rechazada porque la API no exponía imágenes. Catusita agregó el campo 'images' (2026-07-22) y se implementó el mismo día.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(documentos): enviar factura/NC en PDF por WhatsApp (#18)
Conecta el endpoint de documentos electronicos de Catusita:
el vendedor pide la factura o nota de credito de un cliente y Catu
ubica el documento en sus pedidos, descarga el PDF y lo envia al chat.

- tool enviar_documento (RUC-scoped por cartera)
- resolucion tipo_codigo/empresa_codigo desde /pedidos
- send_document_base64 en WAHA y Kapso; webhook distingue foto vs PDF
- solo factura (01) y NC (07), solo PDF (guia de remision no expuesta)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Actualizado: 2026-07-21 16:06 (hora Perú)  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
+          <t>Actualizado: 2026-07-30 (hora Perú)  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
         </is>
       </c>
     </row>
@@ -1077,8 +1077,39 @@
       </c>
       <c r="G21" s="5" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Documentos</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>El agente no podía enviar la factura ni la nota de crédito de un pedido: cuando se lo pedían, avisaba que 'la descarga de documentos todavía no está conectada'. Era una capacidad apagada porque la API de Catusita no exponía los documentos electrónicos.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Catusita expuso el endpoint de documentos electrónicos (búsqueda por N° + tipo + empresa, con URL de PDF/XML). Se conectó al agente: cuando el vendedor pide la factura o la nota de crédito de un cliente, Catu ubica el documento en los pedidos del cliente, descarga el PDF y se lo envía por WhatsApp como archivo. Solo factura (01) y nota de crédito (07), y solo PDF (el XML es para SUNAT/contabilidad). La guía de remisión no está expuesta en este endpoint.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor ya puede pedir la factura o la nota de crédito de un pedido y Catu se la manda al chat como PDF. Antes esto no estaba disponible.</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G21"/>
+  <autoFilter ref="A4:G22"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
feat(cobranzas): estado de pago de una factura/NC por WhatsApp (#19)
Conecta /documento/pagos: el vendedor pregunta si una factura esta pagada,
si se pago con letras o NC, cuanto se debe, y Catu ubica el documento en
los pedidos del cliente y responde estado, saldo y detalle (letras con
vencimiento). tool consultar_pago_documento (scopeada por cartera).
Refactor: _ubicar_documento compartido con enviar_documento.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Actualizado: 2026-07-30 (hora Perú)  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
+          <t>Actualizado: 2026-08-03 (hora Perú)  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
         </is>
       </c>
     </row>
@@ -1108,8 +1108,39 @@
       </c>
       <c r="G22" s="5" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Cobranzas / Documentos</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>El agente no podía decir si una factura estaba pagada, si se había canjeado por letras o si le aplicaron una nota de crédito: la cobranza estaba apagada porque la API de Catusita no lo exponía.</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Catusita expuso el endpoint de aplicación de pagos de documentos. Se conectó al agente: por factura (ubicada en los pedidos del cliente) devuelve el estado de pago, el saldo, si se pagó con letras (con el canje, cada letra y su vencimiento) o con nota de crédito, y el detalle de los pagos. Es el estado de UN documento, no el reporte de cobranzas de toda la cartera (eso sigue apagado). El monto de cada pago se toma de reconciliations[] (el ERP a veces deja el importe del lado del pago en 0).</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor ya puede preguntar '¿esta factura está pagada?' o '¿se pagó con letras?' y Catu le dice el estado, el saldo y el detalle (letras con su vencimiento). Antes no estaba disponible.</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G22"/>
+  <autoFilter ref="A4:G23"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
feat(busqueda): subagente A2A de catalogo (resuelve #20)
Convierte la busqueda de catalogo en un subagente Claude que razona el
termino: ignora año/motor (que rompian el match), prueba sinonimos y
reintenta al dar 0, con fallback determinista. buscar_catalogo delega en
el subagente (drop-in, misma salida).

Verificado: 'filtro para KIA Picanto 2015' -> 4 (antes 0), 'corolla 2018'
-> 6; casos que ya andaban (amortiguador posterior) siguen; parachoques
(inexistente) devuelve 0 sin inventar.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidencias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Incidencias'!$A$4:$G$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +49,12 @@
       <b val="1"/>
       <color rgb="00A61B29"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +74,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,6 +125,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -483,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -505,7 +517,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Actualizado: 2026-08-03 (hora Perú)  ·  Última revisión de chats: 17/07/2026 16:54 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
+          <t>Actualizado: 2026-08-08 (hora Perú)  ·  Última revisión de chats: 07/08/2026 12:49 (hora Perú)  ·  Cada mejora requiere aprobación antes de aplicarse.</t>
         </is>
       </c>
     </row>
@@ -1139,8 +1151,132 @@
       </c>
       <c r="G23" s="5" t="inlineStr"/>
     </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Buscador de catálogo</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Cuando el vendedor agrega el AÑO (ej. 2015, 2018) o el CÓDIGO DE MOTOR (ej. G4LA) al buscar, el catálogo devuelve 0 resultados aunque el producto exista. Caso real (Roger): 'filtro para KIA Picanto 2015' → 0, pero 'filtro de aire picanto' → 4. Confirmado reproduciendo: 'filtro de aire kia picanto' devuelve 4, y al agregar '2015' o 'g4la' cae a 0. También 'filtro aceite corolla 2018' → 0 vs 'filtro aceite corolla' → 6.</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>El buscador exige que TODOS los tokens aparezcan en el producto; el año y el código de motor no están en el texto del artículo, así que rompen el match. Ignorar (o no exigir) los tokens de año (19xx/20xx) y, si el match estricto da 0, reintentar relajando los tokens que por sí solos no matchean ningún producto.</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor podrá buscar como habla ('filtro para Picanto 2015') y el agente igual encontrará el producto, en vez de decir 'no encontré' porque el año o el motor no calzan literalmente.</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Consulta de placa</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Al consultar una placa por Yahuar, además de 'consulta enviada' y los datos finales del vehículo, se le reenvía al vendedor un mensaje intermedio de saludo/aclaración de Yahuar ('¡Hola! Soy Yahuar 😊 ¿qué información buscas sobre esta placa?'). Caso real (Roger, placa BRW527): tras ese mensaje el vendedor respondió 'no ayudas' y recién después llegaron los datos.</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Filtrar los mensajes intermedios de Yahuar (saludo/aclaración) y reenviar al vendedor SOLO los datos finales del vehículo. Ampliar los patrones de aclaración que hoy se descartan (ej. 'qué información buscas', 'veo que me pasas', 'puedo:') o, mejor, reenviar únicamente el bloque estructurado de datos.</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Cuando el vendedor pida una placa, ya no le llegará el saludo de Yahuar que confunde: solo el aviso de 'consultando' y luego los datos del vehículo.</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Cartera de clientes</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Una vendedora (Patricia, 216 clientes) pidió 'envíame mi cartera completa' y el agente respondió que no puede exportar ni enviar un archivo con la lista; solo mostrarla en partes en el chat.</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Permitir exportar la cartera del vendedor como archivo (Excel o PDF) y enviárselo por WhatsApp, igual que hoy se envían las facturas en PDF.</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor podrá pedir su cartera completa y recibir un archivo con todos sus clientes, en vez de tener que verlos por partes en el chat.</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Ventas / Reportes</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Un vendedor (Fernando) pidió 'acumulado de ventas de agosto' y el agente respondió que esa función no está conectada y lo derivó al supervisor.</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Evaluar exponer el acumulado de ventas del vendedor por período (mes). Los montos existen en los pedidos por cliente; habría que agregar un total por vendedor y período (confirmar con Catusita la fuente correcta para no sumar mal facturas/NC).</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>El vendedor podría preguntar cuánto lleva vendido en el mes y el agente le daría el acumulado, en vez de derivarlo al área de ventas.</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G23"/>
+  <autoFilter ref="A4:G27"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
feat(placa): subagente Yahuar bloqueante (resuelve #21)
La consulta de placa deja de ser fire-and-forget: el tool avisa
'consultando', envia la placa y BLOQUEA (en el background task, no cuelga
el HTTP) hasta que el webhook deposita el resultado en Redis, y devuelve
datos limpios + foto para que el agente arme UNA sola respuesta.

- agents/yahuar_subagente.py: envia/bloquea/pollea/devuelve
- shared/yahuar.py: flag bloqueante + resultado en Redis
- webhook _reenviar_yahuar: en modo bloqueante guarda el resultado (no push)
- filtros de saludo/aclaracion de Yahuar ampliados (ya no se cuela)
- kill-switch YAHUAR_BLOQUEANTE=false vuelve al relay async

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -1206,9 +1206,9 @@
           <t>Cuando el vendedor pida una placa, ya no le llegará el saludo de Yahuar que confunde: solo el aviso de 'consultando' y luego los datos del vehículo.</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Aplicado</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(mejoras): #22 y #23 -> Rechazado (no autorizados, en gestion)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mejoras/incidencias.xlsx
+++ b/mejoras/incidencias.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,12 +49,8 @@
       <b val="1"/>
       <color rgb="00A61B29"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C6500"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -74,11 +70,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8D7DA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -108,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -125,9 +116,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1237,12 +1225,16 @@
           <t>El vendedor podrá pedir su cartera completa y recibir un archivo con todos sus clientes, en vez de tener que verlos por partes en el chat.</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr"/>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>No autorizado aún; en gestión. Requiere aprobación antes de implementarse.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -1268,12 +1260,16 @@
           <t>El vendedor podría preguntar cuánto lleva vendido en el mes y el agente le daría el acumulado, en vez de derivarlo al área de ventas.</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr"/>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>No autorizado aún; en gestión. Requiere aprobación antes de implementarse.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:G27"/>

</xml_diff>